<commit_message>
Projectile started,good on serv side
</commit_message>
<xml_diff>
--- a/data/Envoie_données.xlsx
+++ b/data/Envoie_données.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nobil\Unknown\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nobil\Unknown\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C78B7973-B4D4-4CA5-91F7-93EB73A1F893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{501248C4-E3C6-40D4-B890-335B5D18F863}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{B9327B43-8E89-4C75-A473-2C353B32A7CA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
   <si>
     <t>ID send</t>
   </si>
@@ -105,6 +105,12 @@
   </si>
   <si>
     <t>chunk/id/new_pos</t>
+  </si>
+  <si>
+    <t>projectile_create</t>
+  </si>
+  <si>
+    <t>projectile_die</t>
   </si>
 </sst>
 </file>
@@ -476,7 +482,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20C48EE1-EBD0-4B79-91FA-27BBFC80C012}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="3" max="3" width="31.33203125" customWidth="1"/>
@@ -615,6 +621,22 @@
         <v>17</v>
       </c>
     </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="F9">
+        <v>7</v>
+      </c>
+      <c r="G9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="F10">
+        <v>8</v>
+      </c>
+      <c r="G10" t="s">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Can switch spell in weapon
</commit_message>
<xml_diff>
--- a/data/Envoie_données.xlsx
+++ b/data/Envoie_données.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nobil\Unknown\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{137E3614-CCFB-416A-8423-D2E73E762277}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A922F444-7BFD-4EF9-B2A0-33CDE8C5634D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{B9327B43-8E89-4C75-A473-2C353B32A7CA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="34">
   <si>
     <t>ID send</t>
   </si>
@@ -132,6 +132,12 @@
   </si>
   <si>
     <t>id player / new_life</t>
+  </si>
+  <si>
+    <t>Switch spell_pos</t>
+  </si>
+  <si>
+    <t>(weapon/idx)(weapon/idx)</t>
   </si>
 </sst>
 </file>
@@ -507,7 +513,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="3" max="3" width="31.33203125" customWidth="1"/>
-    <col min="4" max="4" width="13.19921875" customWidth="1"/>
+    <col min="4" max="4" width="22.33203125" customWidth="1"/>
     <col min="7" max="7" width="25.73046875" customWidth="1"/>
     <col min="8" max="8" width="28.19921875" customWidth="1"/>
   </cols>
@@ -615,6 +621,15 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" t="s">
+        <v>33</v>
+      </c>
       <c r="F7">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
Can interact with element
</commit_message>
<xml_diff>
--- a/data/Envoie_données.xlsx
+++ b/data/Envoie_données.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nobil\Documents\GithubCode\Unknown\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FECE6DB3-DE76-4823-A3D0-399DB938A444}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{470A863F-036F-463A-BEC4-A3274F014F6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{B9327B43-8E89-4C75-A473-2C353B32A7CA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="49">
   <si>
     <t>ID send</t>
   </si>
@@ -171,6 +171,18 @@
   </si>
   <si>
     <t>id,id_type,pos_x,pos_y,chunk</t>
+  </si>
+  <si>
+    <t>interact with</t>
+  </si>
+  <si>
+    <t>id,chunk of the element</t>
+  </si>
+  <si>
+    <t>Destroy object</t>
+  </si>
+  <si>
+    <t>Chunk,id</t>
   </si>
 </sst>
 </file>
@@ -542,7 +554,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20C48EE1-EBD0-4B79-91FA-27BBFC80C012}">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="3" max="3" width="31.33203125" customWidth="1"/>
@@ -720,6 +732,15 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="B10">
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" t="s">
+        <v>46</v>
+      </c>
       <c r="F10">
         <v>8</v>
       </c>
@@ -799,6 +820,17 @@
       </c>
       <c r="H17" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="6:8" x14ac:dyDescent="0.45">
+      <c r="F18">
+        <v>16</v>
+      </c>
+      <c r="G18" t="s">
+        <v>47</v>
+      </c>
+      <c r="H18" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add spell to inventory
</commit_message>
<xml_diff>
--- a/data/Envoie_données.xlsx
+++ b/data/Envoie_données.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nobil\Documents\GithubCode\Unknown\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{470A863F-036F-463A-BEC4-A3274F014F6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86541B6A-B8FB-4465-8D78-19AAC535CDFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{B9327B43-8E89-4C75-A473-2C353B32A7CA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="51">
   <si>
     <t>ID send</t>
   </si>
@@ -183,6 +183,12 @@
   </si>
   <si>
     <t>Chunk,id</t>
+  </si>
+  <si>
+    <t>Add spell to weapon</t>
+  </si>
+  <si>
+    <t>Id spell, id weapon</t>
   </si>
 </sst>
 </file>
@@ -554,7 +560,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20C48EE1-EBD0-4B79-91FA-27BBFC80C012}">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="3" max="3" width="31.33203125" customWidth="1"/>
@@ -833,6 +839,17 @@
         <v>48</v>
       </c>
     </row>
+    <row r="19" spans="6:8" x14ac:dyDescent="0.45">
+      <c r="F19">
+        <v>17</v>
+      </c>
+      <c r="G19" t="s">
+        <v>49</v>
+      </c>
+      <c r="H19" t="s">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Death on monster done
</commit_message>
<xml_diff>
--- a/data/Envoie_données.xlsx
+++ b/data/Envoie_données.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nobil\Documents\GithubCode\Unknown\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{920A8F10-A7DC-4471-9FB3-F16CBF26105A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72B53C40-0697-4067-B220-ADCDD6B3FE8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{B9327B43-8E89-4C75-A473-2C353B32A7CA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="55">
   <si>
     <t>ID send</t>
   </si>
@@ -195,6 +195,12 @@
   </si>
   <si>
     <t>Idx weapon/idx spell</t>
+  </si>
+  <si>
+    <t>Ent die</t>
+  </si>
+  <si>
+    <t>Id,chunk</t>
   </si>
 </sst>
 </file>
@@ -566,7 +572,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20C48EE1-EBD0-4B79-91FA-27BBFC80C012}">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="3" max="3" width="31.33203125" customWidth="1"/>
@@ -865,6 +871,17 @@
         <v>50</v>
       </c>
     </row>
+    <row r="20" spans="6:8" x14ac:dyDescent="0.45">
+      <c r="F20">
+        <v>18</v>
+      </c>
+      <c r="G20" t="s">
+        <v>53</v>
+      </c>
+      <c r="H20" t="s">
+        <v>54</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add pnj to spawn
</commit_message>
<xml_diff>
--- a/data/Envoie_données.xlsx
+++ b/data/Envoie_données.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nobil\Documents\GithubCode\Unknown\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72B53C40-0697-4067-B220-ADCDD6B3FE8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEE2F7F7-2368-410F-B61E-02D87AB3B757}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{B9327B43-8E89-4C75-A473-2C353B32A7CA}"/>
+    <workbookView xWindow="5280" yWindow="3472" windowWidth="16200" windowHeight="9308" xr2:uid="{B9327B43-8E89-4C75-A473-2C353B32A7CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="56">
   <si>
     <t>ID send</t>
   </si>
@@ -201,6 +201,9 @@
   </si>
   <si>
     <t>Id,chunk</t>
+  </si>
+  <si>
+    <t>TP to boss ?</t>
   </si>
 </sst>
 </file>
@@ -787,6 +790,12 @@
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="B12">
+        <v>10</v>
+      </c>
+      <c r="C12" t="s">
+        <v>55</v>
+      </c>
       <c r="F12">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update many things + Important ! Don't put monster in between chunks !
</commit_message>
<xml_diff>
--- a/data/Envoie_données.xlsx
+++ b/data/Envoie_données.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nobil\Documents\GithubCode\Unknown\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEE2F7F7-2368-410F-B61E-02D87AB3B757}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{909EA495-7AEB-46BD-A744-F00825BC2C1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5280" yWindow="3472" windowWidth="16200" windowHeight="9308" xr2:uid="{B9327B43-8E89-4C75-A473-2C353B32A7CA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="57">
   <si>
     <t>ID send</t>
   </si>
@@ -204,6 +204,9 @@
   </si>
   <si>
     <t>TP to boss ?</t>
+  </si>
+  <si>
+    <t>Too left and didn't talk to pnj</t>
   </si>
 </sst>
 </file>
@@ -575,7 +578,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20C48EE1-EBD0-4B79-91FA-27BBFC80C012}">
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="3" max="3" width="31.33203125" customWidth="1"/>
@@ -891,6 +894,14 @@
         <v>54</v>
       </c>
     </row>
+    <row r="21" spans="6:8" x14ac:dyDescent="0.45">
+      <c r="F21">
+        <v>19</v>
+      </c>
+      <c r="G21" t="s">
+        <v>56</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix speed. + Added pnj double jump
</commit_message>
<xml_diff>
--- a/data/Envoie_données.xlsx
+++ b/data/Envoie_données.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nobil\Documents\GithubCode\Unknown\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{050E6B51-6F1C-488C-8647-0C1CF2A2DADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{495FC19F-3861-4716-AF5B-376067E77174}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4718" yWindow="2813" windowWidth="16200" windowHeight="9307" xr2:uid="{B9327B43-8E89-4C75-A473-2C353B32A7CA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="60">
   <si>
     <t>ID send</t>
   </si>
@@ -213,6 +213,9 @@
   </si>
   <si>
     <t>List : old_chunk / new_chunk / id</t>
+  </si>
+  <si>
+    <t>Debloque double jump</t>
   </si>
 </sst>
 </file>
@@ -816,6 +819,12 @@
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="B13">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
+        <v>59</v>
+      </c>
       <c r="F13">
         <v>11</v>
       </c>

</xml_diff>

<commit_message>
Many fix to have a better experience
</commit_message>
<xml_diff>
--- a/data/Envoie_données.xlsx
+++ b/data/Envoie_données.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nobil\Documents\GithubCode\Unknown\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{495FC19F-3861-4716-AF5B-376067E77174}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60ACA0AA-C4CA-4B70-A77A-CBF6E7A3F22F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4718" yWindow="2813" windowWidth="16200" windowHeight="9307" xr2:uid="{B9327B43-8E89-4C75-A473-2C353B32A7CA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="62">
   <si>
     <t>ID send</t>
   </si>
@@ -216,6 +216,12 @@
   </si>
   <si>
     <t>Debloque double jump</t>
+  </si>
+  <si>
+    <t>Bag full</t>
+  </si>
+  <si>
+    <t>Not enough money to buy</t>
   </si>
 </sst>
 </file>
@@ -587,7 +593,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20C48EE1-EBD0-4B79-91FA-27BBFC80C012}">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="3" max="3" width="31.33203125" customWidth="1"/>
@@ -928,6 +934,22 @@
         <v>58</v>
       </c>
     </row>
+    <row r="23" spans="6:8" x14ac:dyDescent="0.45">
+      <c r="F23">
+        <v>21</v>
+      </c>
+      <c r="G23" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="24" spans="6:8" x14ac:dyDescent="0.45">
+      <c r="F24">
+        <v>22</v>
+      </c>
+      <c r="G24" t="s">
+        <v>61</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix + added alert messages
</commit_message>
<xml_diff>
--- a/data/Envoie_données.xlsx
+++ b/data/Envoie_données.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nobil\Documents\GithubCode\Unknown\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60ACA0AA-C4CA-4B70-A77A-CBF6E7A3F22F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E2EFE83-436E-4228-B871-CEB76798965C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4718" yWindow="2813" windowWidth="16200" windowHeight="9307" xr2:uid="{B9327B43-8E89-4C75-A473-2C353B32A7CA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="64">
   <si>
     <t>ID send</t>
   </si>
@@ -222,6 +222,12 @@
   </si>
   <si>
     <t>Not enough money to buy</t>
+  </si>
+  <si>
+    <t>Reduce time reload</t>
+  </si>
+  <si>
+    <t>Weapon id</t>
   </si>
 </sst>
 </file>
@@ -593,7 +599,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20C48EE1-EBD0-4B79-91FA-27BBFC80C012}">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="3" max="3" width="31.33203125" customWidth="1"/>
@@ -618,9 +624,6 @@
       <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
-        <v>0</v>
-      </c>
       <c r="G1" t="s">
         <v>42</v>
       </c>
@@ -948,6 +951,17 @@
       </c>
       <c r="G24" t="s">
         <v>61</v>
+      </c>
+    </row>
+    <row r="25" spans="6:8" x14ac:dyDescent="0.45">
+      <c r="F25">
+        <v>23</v>
+      </c>
+      <c r="G25" t="s">
+        <v>62</v>
+      </c>
+      <c r="H25" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added wall to upgrade
</commit_message>
<xml_diff>
--- a/data/Envoie_données.xlsx
+++ b/data/Envoie_données.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nobil\Documents\GithubCode\Unknown\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0A56C33-E54C-4867-8EE4-431F78EFC2CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C4726AF-0CF9-4893-B24A-0FC37550171C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4718" yWindow="2813" windowWidth="16200" windowHeight="9307" xr2:uid="{B9327B43-8E89-4C75-A473-2C353B32A7CA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="68">
   <si>
     <t>ID send</t>
   </si>
@@ -234,6 +234,12 @@
   </si>
   <si>
     <t>Alert add life</t>
+  </si>
+  <si>
+    <t>Destoy monster</t>
+  </si>
+  <si>
+    <t>Chunk/id</t>
   </si>
 </sst>
 </file>
@@ -605,7 +611,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20C48EE1-EBD0-4B79-91FA-27BBFC80C012}">
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="3" max="3" width="31.33203125" customWidth="1"/>
@@ -989,6 +995,17 @@
         <v>65</v>
       </c>
     </row>
+    <row r="28" spans="6:8" x14ac:dyDescent="0.45">
+      <c r="F28">
+        <v>26</v>
+      </c>
+      <c r="G28" t="s">
+        <v>66</v>
+      </c>
+      <c r="H28" t="s">
+        <v>67</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Surprise done : )
</commit_message>
<xml_diff>
--- a/data/Envoie_données.xlsx
+++ b/data/Envoie_données.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nobil\Documents\GithubCode\Unknown\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C4726AF-0CF9-4893-B24A-0FC37550171C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20924F38-B8DE-4588-9592-BD755B19D61C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4718" yWindow="2813" windowWidth="16200" windowHeight="9307" xr2:uid="{B9327B43-8E89-4C75-A473-2C353B32A7CA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="70">
   <si>
     <t>ID send</t>
   </si>
@@ -240,6 +240,12 @@
   </si>
   <si>
     <t>Chunk/id</t>
+  </si>
+  <si>
+    <t>Surprise</t>
+  </si>
+  <si>
+    <t>BOSS</t>
   </si>
 </sst>
 </file>
@@ -611,7 +617,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20C48EE1-EBD0-4B79-91FA-27BBFC80C012}">
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="3" max="3" width="31.33203125" customWidth="1"/>
@@ -857,6 +863,12 @@
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="B14">
+        <v>13</v>
+      </c>
+      <c r="C14" t="s">
+        <v>68</v>
+      </c>
       <c r="F14">
         <v>12</v>
       </c>
@@ -1004,6 +1016,22 @@
       </c>
       <c r="H28" t="s">
         <v>67</v>
+      </c>
+    </row>
+    <row r="29" spans="6:8" x14ac:dyDescent="0.45">
+      <c r="F29">
+        <v>27</v>
+      </c>
+      <c r="G29" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="30" spans="6:8" x14ac:dyDescent="0.45">
+      <c r="F30">
+        <v>28</v>
+      </c>
+      <c r="G30" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>